<commit_message>
added mounting holes to pcb
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{240BFB2C-649F-4041-93F2-58CCFF70D8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA66449-69A7-47BD-AB2E-6CFBD6E16E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="55">
   <si>
     <t>Total Cost</t>
   </si>
@@ -125,15 +125,6 @@
     <t>Connect to NI 9221</t>
   </si>
   <si>
-    <t>Arduino Nano Every Microcontroller</t>
-  </si>
-  <si>
-    <t>Every has more RAM than regular Nano</t>
-  </si>
-  <si>
-    <t>ABX00033 Arduino | Embedded MCU, DSP Evaluation Boards | DigiKey</t>
-  </si>
-  <si>
     <t>RC1206FR-071KL YAGEO | Chip Resistor - Surface Mount | DigiKey</t>
   </si>
   <si>
@@ -195,6 +186,21 @@
   </si>
   <si>
     <t>Couldn't find BC550D, but I read BC550CTA is VERY similar. Second vender is part we had in storage (BC547BTF); CTA is higher-gain, low-noise while BTF is mid-gain general purpose.</t>
+  </si>
+  <si>
+    <t>Arduino Nano Microcontroller</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/dfrobot/DFR0010/6588448</t>
+  </si>
+  <si>
+    <t>M4 Screw</t>
+  </si>
+  <si>
+    <t>M4 Washer</t>
+  </si>
+  <si>
+    <t>M4 Hex Nut</t>
   </si>
 </sst>
 </file>
@@ -621,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -632,7 +638,7 @@
     <col min="6" max="6" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="147.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="69.453125" customWidth="1"/>
-    <col min="9" max="9" width="76" customWidth="1"/>
+    <col min="9" max="9" width="45.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="83.54296875" customWidth="1"/>
     <col min="11" max="11" width="62.54296875" customWidth="1"/>
     <col min="12" max="12" width="55.81640625" customWidth="1"/>
@@ -647,10 +653,10 @@
         <v>2</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>3</v>
@@ -702,7 +708,7 @@
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="2"/>
@@ -712,7 +718,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="C3" s="2">
         <v>0</v>
@@ -721,17 +727,15 @@
         <v>1</v>
       </c>
       <c r="E3" s="5">
-        <v>14.9</v>
+        <v>5.9</v>
       </c>
       <c r="F3" s="5">
-        <f t="shared" ref="F3:F11" si="0">E3*D3</f>
-        <v>14.9</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>30</v>
-      </c>
+        <f t="shared" ref="F3:F14" si="0">E3*D3</f>
+        <v>5.9</v>
+      </c>
+      <c r="G3" s="5"/>
       <c r="H3" s="1" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -739,7 +743,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
@@ -755,10 +759,10 @@
         <v>4.72</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -766,7 +770,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
@@ -782,10 +786,10 @@
         <v>12.55</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -840,10 +844,10 @@
         <v>0.2</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -868,10 +872,10 @@
         <v>0.2</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -879,10 +883,10 @@
         <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D9" s="2">
         <v>2</v>
@@ -895,13 +899,13 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
@@ -929,10 +933,10 @@
         <v>4.1399999999999997</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I10" s="4"/>
     </row>
@@ -944,7 +948,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D11" s="2">
         <v>2</v>
@@ -957,83 +961,131 @@
         <v>3.86</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="I11" s="4"/>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="6" t="s">
-        <v>10</v>
-      </c>
+      <c r="E12" s="5"/>
       <c r="F12" s="5">
-        <f>SUM(F2:F11)</f>
-        <v>43.52000000000001</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="G12" s="5"/>
-      <c r="H12" s="3"/>
+      <c r="H12" s="1"/>
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="B13" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
+      <c r="F13" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G13" s="5"/>
-      <c r="H13" s="3"/>
+      <c r="H13" s="1"/>
       <c r="I13" s="4"/>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="B14" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="H14" s="1"/>
+      <c r="I14" s="4"/>
+    </row>
+    <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="E15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="5">
+        <f>SUM(F2:F11)</f>
+        <v>34.519999999999996</v>
+      </c>
+      <c r="G15" s="5"/>
       <c r="H15" s="3"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
       <c r="H16" s="3"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I16" s="4"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="1"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="H6" r:id="rId1" display="https://www.digikey.com/en/products/detail/amphenol-cs-fci/D25S33E4PA00LF/1538080" xr:uid="{CF6559F6-DE29-468F-A8AE-1C573B84539B}"/>
-    <hyperlink ref="H3" r:id="rId2" display="https://www.digikey.com/en/products/detail/arduino/ABX00033/10239972" xr:uid="{E51E5803-9FE0-4C14-AADE-368708EA871F}"/>
+    <hyperlink ref="H3" r:id="rId2" xr:uid="{E51E5803-9FE0-4C14-AADE-368708EA871F}"/>
     <hyperlink ref="H7" r:id="rId3" display="https://www.digikey.com/en/products/detail/yageo/RC1206FR-071KL/728387" xr:uid="{A702FC16-8F83-4E3A-A93F-D9408DD2F39D}"/>
     <hyperlink ref="H8" r:id="rId4" display="https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF1206FT10K0/1759669" xr:uid="{0F8979C0-6DB2-4B44-9FCD-3042501D593A}"/>
     <hyperlink ref="H9" r:id="rId5" display="https://www.digikey.com/en/products/detail/onsemi/BC550CTA/974185" xr:uid="{1C677837-D3CB-4A91-8EDE-D2113FFCBD6D}"/>

</xml_diff>

<commit_message>
update bom and pcb
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA66449-69A7-47BD-AB2E-6CFBD6E16E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7BC9DA-083B-4643-A662-0B03F62ADBEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t>Total Cost</t>
   </si>
@@ -149,9 +149,6 @@
     <t>IRF540NPBF Infineon Technologies | Single FETs, MOSFETs | DigiKey</t>
   </si>
   <si>
-    <t>Need both for complementary pair</t>
-  </si>
-  <si>
     <t>Amount Per Board</t>
   </si>
   <si>
@@ -201,6 +198,18 @@
   </si>
   <si>
     <t>M4 Hex Nut</t>
+  </si>
+  <si>
+    <t>H1, H2, H3</t>
+  </si>
+  <si>
+    <t>H1, H2, H2</t>
+  </si>
+  <si>
+    <t>Need both for complementary pair. P-channel (when gate is lower than source, pulls V up)</t>
+  </si>
+  <si>
+    <t>Need both for complementary pair. N-channel (when gate is higher than source, pulls V down)</t>
   </si>
 </sst>
 </file>
@@ -653,10 +662,10 @@
         <v>2</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>3</v>
@@ -708,7 +717,7 @@
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="2"/>
@@ -718,7 +727,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2">
         <v>0</v>
@@ -735,7 +744,7 @@
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -743,7 +752,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
@@ -759,10 +768,10 @@
         <v>4.72</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -770,7 +779,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
@@ -786,10 +795,10 @@
         <v>12.55</v>
       </c>
       <c r="G5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -886,7 +895,7 @@
         <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D9" s="2">
         <v>2</v>
@@ -899,13 +908,13 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>34</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
@@ -933,7 +942,7 @@
         <v>4.1399999999999997</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>35</v>
@@ -948,7 +957,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" s="2">
         <v>2</v>
@@ -961,7 +970,7 @@
         <v>3.86</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>36</v>
@@ -969,12 +978,16 @@
       <c r="I11" s="4"/>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="B12" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="D12" s="2">
+        <v>3</v>
+      </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5">
         <f t="shared" si="0"/>
@@ -985,12 +998,16 @@
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="D13" s="2">
+        <v>3</v>
+      </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5">
         <f t="shared" si="0"/>
@@ -1003,10 +1020,12 @@
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="D14" s="2">
+        <v>3</v>
+      </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
updated inventory and pcb
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7BC9DA-083B-4643-A662-0B03F62ADBEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DDC2CB-0E90-4BE7-A9D2-AA8506009E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -176,12 +176,6 @@
     <t>BC547BTF onsemi | Single Bipolar Transistors | DigiKey</t>
   </si>
   <si>
-    <t>8 (BTF)</t>
-  </si>
-  <si>
-    <t>0?</t>
-  </si>
-  <si>
     <t>Couldn't find BC550D, but I read BC550CTA is VERY similar. Second vender is part we had in storage (BC547BTF); CTA is higher-gain, low-noise while BTF is mid-gain general purpose.</t>
   </si>
   <si>
@@ -210,6 +204,12 @@
   </si>
   <si>
     <t>Need both for complementary pair. N-channel (when gate is higher than source, pulls V down)</t>
+  </si>
+  <si>
+    <t>8 (BTF), 2 (CTA)</t>
+  </si>
+  <si>
+    <t>Can be swapped with a nano every for a higher ram option</t>
   </si>
 </sst>
 </file>
@@ -727,7 +727,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2">
         <v>0</v>
@@ -742,9 +742,11 @@
         <f t="shared" ref="F3:F14" si="0">E3*D3</f>
         <v>5.9</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="H3" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -755,7 +757,7 @@
         <v>41</v>
       </c>
       <c r="C4" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
@@ -782,7 +784,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2">
         <v>1</v>
@@ -811,7 +813,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2">
         <v>1</v>
@@ -895,7 +897,7 @@
         <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D9" s="2">
         <v>2</v>
@@ -908,7 +910,7 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>34</v>
@@ -929,7 +931,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D10" s="2">
         <v>2</v>
@@ -942,7 +944,7 @@
         <v>4.1399999999999997</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>35</v>
@@ -956,8 +958,8 @@
       <c r="B11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>47</v>
+      <c r="C11" s="2">
+        <v>2</v>
       </c>
       <c r="D11" s="2">
         <v>2</v>
@@ -970,7 +972,7 @@
         <v>3.86</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>36</v>
@@ -979,10 +981,10 @@
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2">
@@ -999,12 +1001,14 @@
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="2"/>
+        <v>50</v>
+      </c>
+      <c r="C13" s="2">
+        <v>12</v>
+      </c>
       <c r="D13" s="2">
         <v>3</v>
       </c>
@@ -1020,9 +1024,11 @@
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="C14" s="2">
+        <v>12</v>
+      </c>
       <c r="D14" s="2">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
updated pcb labels and inventory
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019A76CE-7A73-4DE5-AD87-73D5FE2743C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{415D0405-074B-46BE-A2C9-9877FD8353AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
   <si>
     <t>Total Cost</t>
   </si>
@@ -206,13 +206,16 @@
     <t>Need both for complementary pair. N-channel (when gate is higher than source, pulls V down)</t>
   </si>
   <si>
-    <t>8 (BTF), 2 (CTA)</t>
-  </si>
-  <si>
     <t>Can be swapped with a nano every for a higher ram option</t>
   </si>
   <si>
-    <t>DSUB Screw Retainer Kit</t>
+    <t>6 (BTF), 2 (CTA)</t>
+  </si>
+  <si>
+    <t>DSUB Screw</t>
+  </si>
+  <si>
+    <t>5746879-1 TE Connectivity AMP Connectors | D-Sub, D-Shaped Connector Jackscrews | DigiKey</t>
   </si>
 </sst>
 </file>
@@ -649,7 +652,7 @@
     <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="147.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="69.453125" customWidth="1"/>
+    <col min="8" max="8" width="79" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="45.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="83.54296875" customWidth="1"/>
     <col min="11" max="11" width="62.54296875" customWidth="1"/>
@@ -706,7 +709,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -746,7 +749,7 @@
         <v>5.9</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>48</v>
@@ -816,7 +819,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2">
         <v>1</v>
@@ -845,7 +848,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="2">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D7" s="2">
         <v>2</v>
@@ -873,7 +876,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="2">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D8" s="2">
         <v>2</v>
@@ -900,7 +903,7 @@
         <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9" s="2">
         <v>2</v>
@@ -934,7 +937,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10" s="2">
         <v>2</v>
@@ -962,7 +965,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2">
         <v>2</v>
@@ -1050,20 +1053,22 @@
         <v>58</v>
       </c>
       <c r="C15" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="5">
-        <v>1.96</v>
+        <v>0.59</v>
       </c>
       <c r="F15" s="5">
         <f t="shared" si="0"/>
-        <v>1.96</v>
+        <v>1.18</v>
       </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="1"/>
+      <c r="H15" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="I15" s="4"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1076,7 +1081,7 @@
       </c>
       <c r="F16" s="5">
         <f>SUM(F2:F15)</f>
-        <v>36.479999999999997</v>
+        <v>35.699999999999996</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="3"/>
@@ -1145,8 +1150,9 @@
     <hyperlink ref="H5" r:id="rId9" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757064/260384" xr:uid="{2033BA66-A94C-4F37-8897-CE20B23FC91F}"/>
     <hyperlink ref="H4" r:id="rId10" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757297/260479" xr:uid="{9CCD2936-CC49-4825-A93A-6F99555D80E1}"/>
     <hyperlink ref="I9" r:id="rId11" display="https://www.digikey.com/en/products/detail/onsemi/BC547BTF/976371" xr:uid="{D92774B8-B9A8-4AC5-B1A3-EB1FA0C520CD}"/>
+    <hyperlink ref="H15" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update bom and arduino code
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{415D0405-074B-46BE-A2C9-9877FD8353AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B7E0CEE-9A48-4D18-A3C8-1D9F35F1FFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
   <si>
     <t>Total Cost</t>
   </si>
@@ -216,6 +216,15 @@
   </si>
   <si>
     <t>5746879-1 TE Connectivity AMP Connectors | D-Sub, D-Shaped Connector Jackscrews | DigiKey</t>
+  </si>
+  <si>
+    <t>Power Supply</t>
+  </si>
+  <si>
+    <t>Convenient and plugs into wall</t>
+  </si>
+  <si>
+    <t>GST60A12-P1J MEAN WELL USA Inc. | AC DC Desktop, Wall Power Adapters | DigiKey</t>
   </si>
 </sst>
 </file>
@@ -642,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -745,7 +754,7 @@
         <v>5.9</v>
       </c>
       <c r="F3" s="5">
-        <f t="shared" ref="F3:F15" si="0">E3*D3</f>
+        <f t="shared" ref="F3:F16" si="0">E3*D3</f>
         <v>5.9</v>
       </c>
       <c r="G3" s="5" t="s">
@@ -992,7 +1001,9 @@
       <c r="B12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2">
+        <v>0</v>
+      </c>
       <c r="D12" s="2">
         <v>3</v>
       </c>
@@ -1062,7 +1073,7 @@
         <v>0.59</v>
       </c>
       <c r="F15" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F15" si="1">E15*D15</f>
         <v>1.18</v>
       </c>
       <c r="G15" s="5"/>
@@ -1073,18 +1084,28 @@
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="7" t="s">
-        <v>10</v>
+      <c r="B16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>18.600000000000001</v>
       </c>
       <c r="F16" s="5">
-        <f>SUM(F2:F15)</f>
-        <v>35.699999999999996</v>
-      </c>
-      <c r="G16" s="5"/>
-      <c r="H16" s="3"/>
+        <f t="shared" si="0"/>
+        <v>18.600000000000001</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1092,8 +1113,13 @@
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
+      <c r="E17" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="5">
+        <f>SUM(F2:F16)</f>
+        <v>54.3</v>
+      </c>
       <c r="G17" s="5"/>
       <c r="H17" s="3"/>
       <c r="I17" s="4"/>
@@ -1103,19 +1129,20 @@
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
       <c r="H18" s="3"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I18" s="4"/>
+    </row>
+    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -1130,11 +1157,21 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
-      <c r="H21" s="1"/>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1151,8 +1188,9 @@
     <hyperlink ref="H4" r:id="rId10" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757297/260479" xr:uid="{9CCD2936-CC49-4825-A93A-6F99555D80E1}"/>
     <hyperlink ref="I9" r:id="rId11" display="https://www.digikey.com/en/products/detail/onsemi/BC547BTF/976371" xr:uid="{D92774B8-B9A8-4AC5-B1A3-EB1FA0C520CD}"/>
     <hyperlink ref="H15" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
+    <hyperlink ref="H16" r:id="rId13" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
+  <pageSetup orientation="portrait" r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added mfr part numbers
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D179D32A-F009-4A21-AAF7-B4A0118EEDFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1FD868-D032-4619-9980-D9BE575EA8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
   <si>
     <t>Total Cost</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>5V Barrel Jack</t>
-  </si>
-  <si>
     <t>DSUB-25 Female Connector</t>
   </si>
   <si>
@@ -110,9 +107,6 @@
     <t>Q3, Q5</t>
   </si>
   <si>
-    <t>IRF9540N  HEXFET power MOSFET</t>
-  </si>
-  <si>
     <t>J2 DSUB</t>
   </si>
   <si>
@@ -134,9 +128,6 @@
     <t>Or use resistor book: https://www.adafruit.com/product/442</t>
   </si>
   <si>
-    <t>BC550 Epitaxial Silicon Transistor</t>
-  </si>
-  <si>
     <t>BC550CTA onsemi | Single Bipolar Transistors | DigiKey</t>
   </si>
   <si>
@@ -170,12 +161,6 @@
     <t>1757297 Phoenix Contact | Headers, Plugs and Sockets | DigiKey</t>
   </si>
   <si>
-    <t>BC547BTF onsemi | Single Bipolar Transistors | DigiKey</t>
-  </si>
-  <si>
-    <t>Couldn't find BC550D, but I read BC550CTA is VERY similar. Second vender is part we had in storage (BC547BTF); CTA is higher-gain, low-noise while BTF is mid-gain general purpose.</t>
-  </si>
-  <si>
     <t>Arduino Nano Microcontroller</t>
   </si>
   <si>
@@ -206,9 +191,6 @@
     <t>Can be swapped with a nano every for a higher ram option</t>
   </si>
   <si>
-    <t>6 (BTF), 2 (CTA)</t>
-  </si>
-  <si>
     <t>DSUB Screw</t>
   </si>
   <si>
@@ -224,9 +206,6 @@
     <t>GST60A12-P1J MEAN WELL USA Inc. | AC DC Desktop, Wall Power Adapters | DigiKey</t>
   </si>
   <si>
-    <t>Female Header Pins</t>
-  </si>
-  <si>
     <t>Solder to microcontroller footprint to make detachable</t>
   </si>
   <si>
@@ -236,10 +215,43 @@
     <t>https://www.digikey.com/en/products/detail/amphenol-cs-fci/D25S33E4GX00LF/1001825</t>
   </si>
   <si>
-    <t>Part Number</t>
-  </si>
-  <si>
     <t>D25S33E4GX00LF</t>
+  </si>
+  <si>
+    <t>CTA is higher-gain, low-noise</t>
+  </si>
+  <si>
+    <t>15 Pos Female Header Pins</t>
+  </si>
+  <si>
+    <t>Barrel Jack</t>
+  </si>
+  <si>
+    <t>MFR Part Number</t>
+  </si>
+  <si>
+    <t>PJ-002A</t>
+  </si>
+  <si>
+    <t>RC1206FR-071KL</t>
+  </si>
+  <si>
+    <t>5746879-1</t>
+  </si>
+  <si>
+    <t>RMCF1206FT10K0</t>
+  </si>
+  <si>
+    <t>BC550CTA</t>
+  </si>
+  <si>
+    <t>Epitaxial Silicon Transistor</t>
+  </si>
+  <si>
+    <t>IRF9540NPBF</t>
+  </si>
+  <si>
+    <t>HEXFET power MOSFET</t>
   </si>
 </sst>
 </file>
@@ -667,25 +679,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:N23"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="147.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="147.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="79" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="83.5703125" customWidth="1"/>
-    <col min="12" max="12" width="62.5703125" customWidth="1"/>
-    <col min="13" max="13" width="55.85546875" customWidth="1"/>
+    <col min="10" max="10" width="45.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.54296875" customWidth="1"/>
+    <col min="12" max="12" width="62.54296875" customWidth="1"/>
+    <col min="13" max="13" width="55.81640625" customWidth="1"/>
     <col min="14" max="14" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -693,13 +705,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>3</v>
@@ -729,14 +741,16 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="2"/>
+        <v>62</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="D2" s="2">
         <v>9</v>
       </c>
@@ -752,17 +766,17 @@
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2">
@@ -779,20 +793,22 @@
         <v>5.9</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1757064</v>
+      </c>
       <c r="D4" s="2">
         <v>1</v>
       </c>
@@ -807,20 +823,22 @@
         <v>4.72</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="2"/>
+        <v>36</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1757297</v>
+      </c>
       <c r="D5" s="2">
         <v>1</v>
       </c>
@@ -835,23 +853,23 @@
         <v>12.55</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D6" s="2">
         <v>0</v>
@@ -867,22 +885,24 @@
         <v>1.81</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J6" s="3"/>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="D7" s="2">
         <v>48</v>
       </c>
@@ -897,21 +917,23 @@
         <v>0.2</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="D8" s="2">
         <v>48</v>
       </c>
@@ -926,22 +948,24 @@
         <v>0.2</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
-        <v>56</v>
+        <v>69</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2</v>
       </c>
       <c r="E9" s="2">
         <v>2</v>
@@ -954,27 +978,27 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>44</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="J9" s="1"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="D10" s="2">
         <v>7</v>
       </c>
@@ -989,19 +1013,19 @@
         <v>4.1399999999999997</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2">
@@ -1018,19 +1042,19 @@
         <v>3.86</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2">
@@ -1048,12 +1072,12 @@
       <c r="I12" s="1"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2">
@@ -1071,10 +1095,10 @@
       <c r="I13" s="1"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2">
@@ -1092,12 +1116,14 @@
       <c r="I14" s="1"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="D15" s="2">
         <v>0</v>
       </c>
@@ -1113,14 +1139,14 @@
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2">
@@ -1137,17 +1163,17 @@
         <v>11.72</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="J16" s="4"/>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2">
@@ -1164,14 +1190,14 @@
         <v>18.600000000000001</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1188,7 +1214,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1200,7 +1226,7 @@
       <c r="I19" s="3"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1211,7 +1237,7 @@
       <c r="H20" s="5"/>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1222,7 +1248,7 @@
       <c r="H21" s="2"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1233,7 +1259,7 @@
       <c r="H22" s="2"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -1253,13 +1279,12 @@
     <hyperlink ref="I2" r:id="rId7" display="https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/PJ-002A/96962" xr:uid="{568D8FFB-A50B-4C55-ADF3-BEF9ED909CF8}"/>
     <hyperlink ref="I5" r:id="rId8" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757064/260384" xr:uid="{2033BA66-A94C-4F37-8897-CE20B23FC91F}"/>
     <hyperlink ref="I4" r:id="rId9" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757297/260479" xr:uid="{9CCD2936-CC49-4825-A93A-6F99555D80E1}"/>
-    <hyperlink ref="J9" r:id="rId10" display="https://www.digikey.com/en/products/detail/onsemi/BC547BTF/976371" xr:uid="{D92774B8-B9A8-4AC5-B1A3-EB1FA0C520CD}"/>
-    <hyperlink ref="I15" r:id="rId11" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
-    <hyperlink ref="I17" r:id="rId12" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
-    <hyperlink ref="I16" r:id="rId13" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
-    <hyperlink ref="I6" r:id="rId14" xr:uid="{9DD314B7-3D79-461E-9C6A-997EEC8DC3BE}"/>
+    <hyperlink ref="I15" r:id="rId10" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
+    <hyperlink ref="I17" r:id="rId11" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
+    <hyperlink ref="I16" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
+    <hyperlink ref="I6" r:id="rId13" xr:uid="{9DD314B7-3D79-461E-9C6A-997EEC8DC3BE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId15"/>
+  <pageSetup orientation="portrait" r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updates to box assembly and added screws to BOM
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e6d0746713a8929/Documents/GitHub/Biphasic-data-acquisition-system/DAQ_design/Assisi/v0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1FD868-D032-4619-9980-D9BE575EA8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{5D1FD868-D032-4619-9980-D9BE575EA8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C78C0CA0-C4EB-4264-A010-C73094A7B17E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="77">
   <si>
     <t>Total Cost</t>
   </si>
@@ -252,6 +252,21 @@
   </si>
   <si>
     <t>HEXFET power MOSFET</t>
+  </si>
+  <si>
+    <t>M4 x 40 mm Socket Head Cap Screw</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Socket-Head-Cap-Screw-M4x0-6DB37</t>
+  </si>
+  <si>
+    <t>6DB37</t>
+  </si>
+  <si>
+    <t>Package quantity 50</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Socket-Head-Cap-Screw-M4x0-22UD47</t>
   </si>
 </sst>
 </file>
@@ -678,26 +693,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:N23"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="147.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="147.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="79" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="83.54296875" customWidth="1"/>
-    <col min="12" max="12" width="62.54296875" customWidth="1"/>
-    <col min="13" max="13" width="55.81640625" customWidth="1"/>
+    <col min="10" max="10" width="45.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.5546875" customWidth="1"/>
+    <col min="12" max="12" width="62.5546875" customWidth="1"/>
+    <col min="13" max="13" width="55.77734375" customWidth="1"/>
     <col min="14" max="14" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -741,7 +756,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -771,7 +786,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -789,7 +804,7 @@
         <v>5.9</v>
       </c>
       <c r="G3" s="5">
-        <f t="shared" ref="G3:G17" si="0">F3*E3</f>
+        <f t="shared" ref="G3:G18" si="0">F3*E3</f>
         <v>5.9</v>
       </c>
       <c r="H3" s="5" t="s">
@@ -799,7 +814,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -829,7 +844,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -861,7 +876,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -893,7 +908,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -924,7 +939,7 @@
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -954,7 +969,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -989,7 +1004,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -1020,7 +1035,7 @@
       </c>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
@@ -1049,7 +1064,7 @@
       </c>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>47</v>
       </c>
@@ -1072,7 +1087,7 @@
       <c r="I12" s="1"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>46</v>
       </c>
@@ -1095,60 +1110,66 @@
       <c r="I13" s="1"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>74</v>
+      </c>
       <c r="D14" s="2">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2">
-        <v>3</v>
-      </c>
-      <c r="F14" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="F14" s="5">
+        <v>10.31</v>
+      </c>
       <c r="G14" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="4"/>
-    </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>10.31</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="C15" s="2"/>
       <c r="D15" s="2">
+        <v>12</v>
+      </c>
+      <c r="E15" s="2">
+        <v>3</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E15" s="2">
-        <v>2</v>
-      </c>
-      <c r="F15" s="5">
-        <v>0.59</v>
-      </c>
-      <c r="G15" s="5">
-        <f t="shared" ref="G15" si="1">F15*E15</f>
-        <v>1.18</v>
-      </c>
       <c r="H15" s="5"/>
-      <c r="I15" s="1" t="s">
-        <v>52</v>
-      </c>
+      <c r="I15" s="1"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="D16" s="2">
         <v>0</v>
       </c>
@@ -1156,99 +1177,113 @@
         <v>2</v>
       </c>
       <c r="F16" s="5">
-        <v>5.86</v>
+        <v>0.59</v>
       </c>
       <c r="G16" s="5">
-        <f t="shared" ref="G16" si="2">F16*E16</f>
-        <v>11.72</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>56</v>
-      </c>
+        <f t="shared" ref="G16" si="1">F16*E16</f>
+        <v>1.18</v>
+      </c>
+      <c r="H16" s="5"/>
       <c r="I16" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="J16" s="4"/>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2">
         <v>0</v>
       </c>
       <c r="E17" s="2">
+        <v>2</v>
+      </c>
+      <c r="F17" s="5">
+        <v>5.86</v>
+      </c>
+      <c r="G17" s="5">
+        <f t="shared" ref="G17" si="2">F17*E17</f>
+        <v>11.72</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J17" s="4"/>
+    </row>
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2">
         <v>1</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F18" s="5">
         <v>18.600000000000001</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G18" s="5">
         <f t="shared" si="0"/>
         <v>18.600000000000001</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H18" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="J17" s="4"/>
-    </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="5">
-        <f>SUM(G2:G17)</f>
-        <v>66.02</v>
-      </c>
-      <c r="H18" s="5"/>
-      <c r="I18" s="3"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="F19" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="5">
+        <f>SUM(G2:G18)</f>
+        <v>76.33</v>
+      </c>
       <c r="H19" s="5"/>
       <c r="I19" s="3"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="F20" s="5"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="J20" s="4"/>
+    </row>
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1259,13 +1294,24 @@
       <c r="H22" s="2"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
-      <c r="I23" s="1"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1279,12 +1325,14 @@
     <hyperlink ref="I2" r:id="rId7" display="https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/PJ-002A/96962" xr:uid="{568D8FFB-A50B-4C55-ADF3-BEF9ED909CF8}"/>
     <hyperlink ref="I5" r:id="rId8" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757064/260384" xr:uid="{2033BA66-A94C-4F37-8897-CE20B23FC91F}"/>
     <hyperlink ref="I4" r:id="rId9" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757297/260479" xr:uid="{9CCD2936-CC49-4825-A93A-6F99555D80E1}"/>
-    <hyperlink ref="I15" r:id="rId10" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
-    <hyperlink ref="I17" r:id="rId11" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
-    <hyperlink ref="I16" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
+    <hyperlink ref="I16" r:id="rId10" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
+    <hyperlink ref="I18" r:id="rId11" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
+    <hyperlink ref="I17" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
     <hyperlink ref="I6" r:id="rId13" xr:uid="{9DD314B7-3D79-461E-9C6A-997EEC8DC3BE}"/>
+    <hyperlink ref="I14" r:id="rId14" xr:uid="{7FB61CC9-F2C1-46B2-AF32-B41433DD34B1}"/>
+    <hyperlink ref="J14" r:id="rId15" xr:uid="{D978D96B-76FE-4235-B48B-FC9603ECDD3C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated M4 x 40 mm screw link BOM
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e6d0746713a8929/Documents/GitHub/Biphasic-data-acquisition-system/DAQ_design/Assisi/v0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{5D1FD868-D032-4619-9980-D9BE575EA8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C78C0CA0-C4EB-4264-A010-C73094A7B17E}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{5D1FD868-D032-4619-9980-D9BE575EA8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59B30E0D-D91F-4508-87D1-E3F38BAB3730}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="76">
   <si>
     <t>Total Cost</t>
   </si>
@@ -264,9 +264,6 @@
   </si>
   <si>
     <t>Package quantity 50</t>
-  </si>
-  <si>
-    <t>https://www.grainger.com/product/Socket-Head-Cap-Screw-M4x0-22UD47</t>
   </si>
 </sst>
 </file>
@@ -1137,9 +1134,6 @@
       <c r="I14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="J14" s="3" t="s">
-        <v>76</v>
-      </c>
     </row>
     <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
@@ -1160,7 +1154,7 @@
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="4"/>
+      <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -1330,9 +1324,8 @@
     <hyperlink ref="I17" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
     <hyperlink ref="I6" r:id="rId13" xr:uid="{9DD314B7-3D79-461E-9C6A-997EEC8DC3BE}"/>
     <hyperlink ref="I14" r:id="rId14" xr:uid="{7FB61CC9-F2C1-46B2-AF32-B41433DD34B1}"/>
-    <hyperlink ref="J14" r:id="rId15" xr:uid="{D978D96B-76FE-4235-B48B-FC9603ECDD3C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId16"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated M4 hex nut link - Grainger
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adowney2\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e6d0746713a8929/Documents/GitHub/Biphasic-data-acquisition-system/DAQ_design/Assisi/v0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E51C6B-E5C5-4586-A688-9E1075DE122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{B7E51C6B-E5C5-4586-A688-9E1075DE122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51B4DA29-66E9-4469-97BC-D9B3DD60FA8A}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-6540" windowWidth="16440" windowHeight="28320" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="93">
   <si>
     <t>Total Cost</t>
   </si>
@@ -312,6 +312,9 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A09-P1J/7703711</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Hex-Nut-Std-Hex-22UK82</t>
   </si>
 </sst>
 </file>
@@ -739,25 +742,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:N31"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="147.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="147.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="79" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="83.5703125" customWidth="1"/>
-    <col min="12" max="12" width="62.5703125" customWidth="1"/>
-    <col min="13" max="13" width="55.85546875" customWidth="1"/>
+    <col min="10" max="10" width="45.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.5546875" customWidth="1"/>
+    <col min="12" max="12" width="62.5546875" customWidth="1"/>
+    <col min="13" max="13" width="55.88671875" customWidth="1"/>
     <col min="14" max="14" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -801,7 +804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -831,7 +834,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -859,7 +862,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -889,7 +892,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -921,7 +924,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -951,7 +954,7 @@
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -983,7 +986,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1014,7 +1017,7 @@
       </c>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1044,7 +1047,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -1079,7 +1082,7 @@
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
@@ -1110,7 +1113,7 @@
       </c>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -1139,7 +1142,7 @@
       </c>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>47</v>
       </c>
@@ -1162,7 +1165,7 @@
       <c r="I13" s="1"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1185,7 +1188,7 @@
       <c r="I14" s="1"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
         <v>71</v>
@@ -1213,7 +1216,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>45</v>
@@ -1231,10 +1234,12 @@
         <v>0</v>
       </c>
       <c r="H16" s="5"/>
-      <c r="I16" s="1"/>
+      <c r="I16" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
         <v>51</v>
@@ -1261,7 +1266,7 @@
       </c>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
         <v>60</v>
@@ -1288,7 +1293,7 @@
       </c>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
         <v>75</v>
@@ -1315,7 +1320,7 @@
       </c>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
         <v>75</v>
@@ -1339,7 +1344,7 @@
       </c>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="2" t="s">
         <v>79</v>
       </c>
@@ -1367,7 +1372,7 @@
       </c>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="2" t="s">
         <v>82</v>
       </c>
@@ -1393,7 +1398,7 @@
       </c>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
         <v>83</v>
       </c>
@@ -1416,7 +1421,7 @@
       </c>
       <c r="J23" s="4"/>
     </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
         <v>84</v>
       </c>
@@ -1439,7 +1444,7 @@
       </c>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
         <v>85</v>
       </c>
@@ -1462,7 +1467,7 @@
       </c>
       <c r="J25" s="4"/>
     </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1479,7 +1484,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="4"/>
     </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1491,7 +1496,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="4"/>
     </row>
-    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1502,7 +1507,7 @@
       <c r="H28" s="5"/>
       <c r="I28" s="3"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1513,7 +1518,7 @@
       <c r="H29" s="2"/>
       <c r="I29" s="3"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1524,7 +1529,7 @@
       <c r="H30" s="2"/>
       <c r="I30" s="3"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
@@ -1556,8 +1561,9 @@
     <hyperlink ref="I24" r:id="rId19" xr:uid="{C76A3930-6E7E-4232-B1F1-2ED5A173BA06}"/>
     <hyperlink ref="I22" r:id="rId20" xr:uid="{89930E83-4AEA-4DE5-8019-E1271D4CE40C}"/>
     <hyperlink ref="I20" r:id="rId21" xr:uid="{2D3AA0A6-0D92-4AA2-9646-17F5F35EE4DB}"/>
+    <hyperlink ref="I16" r:id="rId22" xr:uid="{40199BE7-DAC8-4F2F-B423-BBE8840267EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId23"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
m4 washer vendor added - grainger
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e6d0746713a8929/Documents/GitHub/Biphasic-data-acquisition-system/DAQ_design/Assisi/v0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{B7E51C6B-E5C5-4586-A688-9E1075DE122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51B4DA29-66E9-4469-97BC-D9B3DD60FA8A}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{B7E51C6B-E5C5-4586-A688-9E1075DE122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BC45980-0ED4-43C7-8F02-A19FF70D94C9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="94">
   <si>
     <t>Total Cost</t>
   </si>
@@ -315,6 +315,9 @@
   </si>
   <si>
     <t>https://www.grainger.com/product/Hex-Nut-Std-Hex-22UK82</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Flat-Washer-18-8-895Y45</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1188,9 @@
         <v>0</v>
       </c>
       <c r="H14" s="5"/>
-      <c r="I14" s="1"/>
+      <c r="I14" s="1" t="s">
+        <v>93</v>
+      </c>
       <c r="J14" s="4"/>
     </row>
     <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1562,8 +1567,9 @@
     <hyperlink ref="I22" r:id="rId20" xr:uid="{89930E83-4AEA-4DE5-8019-E1271D4CE40C}"/>
     <hyperlink ref="I20" r:id="rId21" xr:uid="{2D3AA0A6-0D92-4AA2-9646-17F5F35EE4DB}"/>
     <hyperlink ref="I16" r:id="rId22" xr:uid="{40199BE7-DAC8-4F2F-B423-BBE8840267EA}"/>
+    <hyperlink ref="I14" r:id="rId23" xr:uid="{C2CB1F68-7DA6-4977-9886-3337AFE63AE3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId23"/>
+  <pageSetup orientation="portrait" r:id="rId24"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
M4 x 16 mm socket head cap screw
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e6d0746713a8929/Documents/GitHub/Biphasic-data-acquisition-system/DAQ_design/Assisi/v0.2.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{B7E51C6B-E5C5-4586-A688-9E1075DE122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BC45980-0ED4-43C7-8F02-A19FF70D94C9}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{B7E51C6B-E5C5-4586-A688-9E1075DE122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CFCF6B5-25CD-465A-9D54-B0D6C5B876A6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="96">
   <si>
     <t>Total Cost</t>
   </si>
@@ -317,7 +317,13 @@
     <t>https://www.grainger.com/product/Hex-Nut-Std-Hex-22UK82</t>
   </si>
   <si>
-    <t>https://www.grainger.com/product/Flat-Washer-18-8-895Y45</t>
+    <t>https://nam02.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.grainger.com%2Fproduct%2FFlat-Washer-18-8-26WC32&amp;data=05%7C02%7CAIGIESE%40email.sc.edu%7Cf05aada4311643fb699908ded0976258%7C4b2a4b19d135420e8bb2b1cd238998cc%7C0%7C0%7C639177545789061167%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=6CoqYV%2BZ3hTIH8hXzw%2B6eFP6vmT5tDuPQxYZMFG%2B9QQ%3D&amp;reserved=0</t>
+  </si>
+  <si>
+    <t>M4 x 16 mm Socket Head Cap Screw</t>
+  </si>
+  <si>
+    <t>https://www.grainger.com/product/Socket-Head-Cap-Screw-M4x0-22UC47</t>
   </si>
 </sst>
 </file>
@@ -744,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
@@ -855,7 +861,7 @@
         <v>5.9</v>
       </c>
       <c r="G3" s="5">
-        <f t="shared" ref="G3:G22" si="0">F3*E3</f>
+        <f t="shared" ref="G3:G23" si="0">F3*E3</f>
         <v>5.9</v>
       </c>
       <c r="H3" s="5" t="s">
@@ -1224,104 +1230,92 @@
     <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="C16" s="2"/>
-      <c r="D16" s="2">
-        <v>12</v>
-      </c>
-      <c r="E16" s="2">
-        <v>3</v>
-      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="J16" s="3"/>
+        <v>95</v>
+      </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>65</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="C17" s="2"/>
       <c r="D17" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E17" s="2">
-        <v>2</v>
-      </c>
-      <c r="F17" s="5">
-        <v>0.59</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="F17" s="5"/>
       <c r="G17" s="5">
-        <f t="shared" ref="G17" si="1">F17*E17</f>
-        <v>1.18</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J17" s="4"/>
+        <v>92</v>
+      </c>
+      <c r="J17" s="3"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E18" s="2">
         <v>2</v>
       </c>
       <c r="F18" s="5">
-        <v>5.86</v>
+        <v>0.59</v>
       </c>
       <c r="G18" s="5">
-        <f t="shared" ref="G18" si="2">F18*E18</f>
-        <v>11.72</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>55</v>
-      </c>
+        <f t="shared" ref="G18" si="1">F18*E18</f>
+        <v>1.18</v>
+      </c>
+      <c r="H18" s="5"/>
       <c r="I18" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="J18" s="4"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="5">
-        <v>18.600000000000001</v>
+        <v>5.86</v>
       </c>
       <c r="G19" s="5">
-        <f t="shared" si="0"/>
-        <v>18.600000000000001</v>
+        <f t="shared" ref="G19" si="2">F19*E19</f>
+        <v>11.72</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J19" s="4"/>
     </row>
@@ -1340,22 +1334,24 @@
       <c r="F20" s="5">
         <v>18.600000000000001</v>
       </c>
-      <c r="G20" s="5"/>
+      <c r="G20" s="5">
+        <f t="shared" si="0"/>
+        <v>18.600000000000001</v>
+      </c>
       <c r="H20" s="5" t="s">
         <v>53</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="J20" s="4"/>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>80</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C21" s="2"/>
       <c r="D21" s="2">
         <v>1</v>
       </c>
@@ -1363,52 +1359,51 @@
         <v>1</v>
       </c>
       <c r="F21" s="5">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+      <c r="F22" s="5">
         <v>65.510000000000005</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G22" s="5">
         <f t="shared" si="0"/>
         <v>65.510000000000005</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="H22" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C22" s="2">
-        <v>3200519</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2">
-        <v>2</v>
-      </c>
-      <c r="F22" s="5">
-        <v>0.15</v>
-      </c>
-      <c r="G22" s="5">
-        <f t="shared" si="0"/>
-        <v>0.3</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C23" s="2">
-        <v>3201097</v>
+        <v>3200519</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2">
@@ -1417,21 +1412,24 @@
       <c r="F23" s="5">
         <v>0.15</v>
       </c>
-      <c r="G23" s="5"/>
+      <c r="G23" s="5">
+        <f t="shared" si="0"/>
+        <v>0.3</v>
+      </c>
       <c r="H23" s="5" t="s">
         <v>90</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C24" s="2">
-        <v>3201110</v>
+        <v>3201097</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2">
@@ -1445,16 +1443,16 @@
         <v>90</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C25" s="2">
-        <v>3200904</v>
+        <v>3201110</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2">
@@ -1468,25 +1466,31 @@
         <v>90</v>
       </c>
       <c r="I25" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="2">
+        <v>3200904</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2">
+        <v>2</v>
+      </c>
+      <c r="F26" s="5">
+        <v>0.15</v>
+      </c>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="J25" s="4"/>
-    </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="5">
-        <f>SUM(G2:G22)</f>
-        <v>151.64000000000004</v>
-      </c>
-      <c r="H26" s="5"/>
-      <c r="I26" s="3"/>
       <c r="J26" s="4"/>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1495,8 +1499,13 @@
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
+      <c r="F27" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="5">
+        <f>SUM(G2:G23)</f>
+        <v>151.64000000000004</v>
+      </c>
       <c r="H27" s="5"/>
       <c r="I27" s="3"/>
       <c r="J27" s="4"/>
@@ -1507,20 +1516,21 @@
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
+      <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
       <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
       <c r="I29" s="3"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
@@ -1536,11 +1546,22 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="1"/>
+      <c r="I31" s="3"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1554,22 +1575,23 @@
     <hyperlink ref="I2" r:id="rId7" display="https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/PJ-002A/96962" xr:uid="{568D8FFB-A50B-4C55-ADF3-BEF9ED909CF8}"/>
     <hyperlink ref="I5" r:id="rId8" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757064/260384" xr:uid="{2033BA66-A94C-4F37-8897-CE20B23FC91F}"/>
     <hyperlink ref="I4" r:id="rId9" display="https://www.digikey.com/en/products/detail/phoenix-contact/1757297/260479" xr:uid="{9CCD2936-CC49-4825-A93A-6F99555D80E1}"/>
-    <hyperlink ref="I17" r:id="rId10" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
-    <hyperlink ref="I19" r:id="rId11" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
-    <hyperlink ref="I18" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
+    <hyperlink ref="I18" r:id="rId10" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/5746879-1/2259521?so=99129841&amp;content=productdetail_row&amp;mkt_tok=MDI4LVNYSy01MDcAAAGhrFahbx9pi1nb6U1_s4a7w7WS1p3X3INFI0ss_GDSarh_0yxAQI_ou7h33vsiRGqzkAi1tRJ_RMrPOqZNoaK887jiuNeK_w3vjsVex_a8hJ4" xr:uid="{BDE66ED6-EDAE-4753-B79E-825610EEE962}"/>
+    <hyperlink ref="I20" r:id="rId11" display="https://www.digikey.com/en/products/detail/mean-well-usa-inc/GST60A12-P1J/7703712" xr:uid="{78CD07DF-07E7-4658-BB2C-F43FEF69A3FE}"/>
+    <hyperlink ref="I19" r:id="rId12" display="https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/1-215297-5/5589672?s=N4IgjCBcoEwBxVAYygMwIYBsDOBTANCAPZQDaIAzAJwxUBsADCALqEAOALlCAMocBOASwB2AcxABfQnATQQKSBhwFiZEFQDsAVjAUW7LpF4CR4qSB0xE8tFjyESkchQAsdLe-0hO3PkLGShAC0VnIKAgCuKo7kWiwS5qHkABa46AAmuPwABGwi2PFAA" xr:uid="{D892475B-FE55-4130-9723-35E629B254E7}"/>
     <hyperlink ref="I7" r:id="rId13" xr:uid="{9DD314B7-3D79-461E-9C6A-997EEC8DC3BE}"/>
     <hyperlink ref="I15" r:id="rId14" xr:uid="{7FB61CC9-F2C1-46B2-AF32-B41433DD34B1}"/>
     <hyperlink ref="I6" r:id="rId15" xr:uid="{3915B292-27C3-4E7F-86DE-77131ED779EF}"/>
-    <hyperlink ref="I21" r:id="rId16" xr:uid="{40ADA453-3DCA-42C1-8201-B866A4C3206E}"/>
-    <hyperlink ref="I23" r:id="rId17" xr:uid="{2332F781-0981-412B-8087-9EF083A34C09}"/>
-    <hyperlink ref="I25" r:id="rId18" xr:uid="{9D4C7BC7-8534-4598-B66B-9F4B7BF124CC}"/>
-    <hyperlink ref="I24" r:id="rId19" xr:uid="{C76A3930-6E7E-4232-B1F1-2ED5A173BA06}"/>
-    <hyperlink ref="I22" r:id="rId20" xr:uid="{89930E83-4AEA-4DE5-8019-E1271D4CE40C}"/>
-    <hyperlink ref="I20" r:id="rId21" xr:uid="{2D3AA0A6-0D92-4AA2-9646-17F5F35EE4DB}"/>
-    <hyperlink ref="I16" r:id="rId22" xr:uid="{40199BE7-DAC8-4F2F-B423-BBE8840267EA}"/>
-    <hyperlink ref="I14" r:id="rId23" xr:uid="{C2CB1F68-7DA6-4977-9886-3337AFE63AE3}"/>
+    <hyperlink ref="I22" r:id="rId16" xr:uid="{40ADA453-3DCA-42C1-8201-B866A4C3206E}"/>
+    <hyperlink ref="I24" r:id="rId17" xr:uid="{2332F781-0981-412B-8087-9EF083A34C09}"/>
+    <hyperlink ref="I26" r:id="rId18" xr:uid="{9D4C7BC7-8534-4598-B66B-9F4B7BF124CC}"/>
+    <hyperlink ref="I25" r:id="rId19" xr:uid="{C76A3930-6E7E-4232-B1F1-2ED5A173BA06}"/>
+    <hyperlink ref="I23" r:id="rId20" xr:uid="{89930E83-4AEA-4DE5-8019-E1271D4CE40C}"/>
+    <hyperlink ref="I21" r:id="rId21" xr:uid="{2D3AA0A6-0D92-4AA2-9646-17F5F35EE4DB}"/>
+    <hyperlink ref="I17" r:id="rId22" xr:uid="{40199BE7-DAC8-4F2F-B423-BBE8840267EA}"/>
+    <hyperlink ref="I14" r:id="rId23" display="https://nam02.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.grainger.com%2Fproduct%2FFlat-Washer-18-8-26WC32&amp;data=05%7C02%7CAIGIESE%40email.sc.edu%7Cf05aada4311643fb699908ded0976258%7C4b2a4b19d135420e8bb2b1cd238998cc%7C0%7C0%7C639177545789061167%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=6CoqYV%2BZ3hTIH8hXzw%2B6eFP6vmT5tDuPQxYZMFG%2B9QQ%3D&amp;reserved=0" xr:uid="{E2FAF909-C6EC-4B0D-91E7-8D4FC250EEF3}"/>
+    <hyperlink ref="I16" r:id="rId24" xr:uid="{35C9B14E-1DDC-4ADE-A779-D46ACC35493F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId24"/>
+  <pageSetup orientation="portrait" r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update BOM and added notes
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slm30\Documents\GitHub\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF89D4B1-DE6B-4193-BF5A-B0B56A726489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB5C1F7-91CE-48FC-B3EA-504CDA2E5B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="111">
   <si>
     <t>Total Cost</t>
   </si>
@@ -366,6 +366,9 @@
   </si>
   <si>
     <t>NI 9171 781425-01</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/encore-wire/76502-18-01/2758161</t>
   </si>
 </sst>
 </file>
@@ -793,25 +796,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:N34"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="147.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="147.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="79" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="83.54296875" customWidth="1"/>
-    <col min="12" max="12" width="62.54296875" customWidth="1"/>
-    <col min="13" max="13" width="55.81640625" customWidth="1"/>
+    <col min="10" max="10" width="45.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.5703125" customWidth="1"/>
+    <col min="12" max="12" width="62.5703125" customWidth="1"/>
+    <col min="13" max="13" width="55.85546875" customWidth="1"/>
     <col min="14" max="14" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -855,7 +858,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -885,7 +888,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -913,7 +916,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -943,7 +946,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -975,7 +978,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1007,7 +1010,7 @@
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1039,7 +1042,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1070,7 +1073,7 @@
       </c>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1100,7 +1103,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -1135,7 +1138,7 @@
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -1166,7 +1169,7 @@
       </c>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
@@ -1195,7 +1198,7 @@
       </c>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -1227,7 +1230,7 @@
       </c>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
         <v>67</v>
@@ -1256,7 +1259,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
         <v>89</v>
@@ -1285,7 +1288,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>42</v>
@@ -1315,7 +1318,7 @@
       </c>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
         <v>47</v>
@@ -1342,7 +1345,7 @@
       </c>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
         <v>56</v>
@@ -1369,7 +1372,7 @@
       </c>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
         <v>104</v>
@@ -1396,7 +1399,7 @@
       </c>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
         <v>71</v>
@@ -1423,7 +1426,7 @@
       </c>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>75</v>
       </c>
@@ -1447,11 +1450,11 @@
         <v>77</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
         <v>78</v>
       </c>
@@ -1479,7 +1482,7 @@
       </c>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
         <v>79</v>
       </c>
@@ -1507,7 +1510,7 @@
       </c>
       <c r="J23" s="4"/>
     </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
         <v>80</v>
       </c>
@@ -1535,7 +1538,7 @@
       </c>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>81</v>
       </c>
@@ -1563,7 +1566,7 @@
       </c>
       <c r="J25" s="4"/>
     </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>92</v>
       </c>
@@ -1593,7 +1596,7 @@
       </c>
       <c r="J26" s="4"/>
     </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
         <v>105</v>
       </c>
@@ -1619,7 +1622,7 @@
       </c>
       <c r="J27" s="4"/>
     </row>
-    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
         <v>107</v>
       </c>
@@ -1643,7 +1646,7 @@
       <c r="I28" s="1"/>
       <c r="J28" s="4"/>
     </row>
-    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1660,7 +1663,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="4"/>
     </row>
-    <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1672,7 +1675,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="4"/>
     </row>
-    <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1683,7 +1686,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="3"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1694,7 +1697,7 @@
       <c r="H32" s="2"/>
       <c r="I32" s="3"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1705,7 +1708,7 @@
       <c r="H33" s="2"/>
       <c r="I33" s="3"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -1731,19 +1734,18 @@
     <hyperlink ref="I7" r:id="rId13" xr:uid="{9DD314B7-3D79-461E-9C6A-997EEC8DC3BE}"/>
     <hyperlink ref="I14" r:id="rId14" xr:uid="{7FB61CC9-F2C1-46B2-AF32-B41433DD34B1}"/>
     <hyperlink ref="I6" r:id="rId15" xr:uid="{3915B292-27C3-4E7F-86DE-77131ED779EF}"/>
-    <hyperlink ref="I21" r:id="rId16" xr:uid="{40ADA453-3DCA-42C1-8201-B866A4C3206E}"/>
-    <hyperlink ref="I23" r:id="rId17" xr:uid="{2332F781-0981-412B-8087-9EF083A34C09}"/>
-    <hyperlink ref="I25" r:id="rId18" xr:uid="{9D4C7BC7-8534-4598-B66B-9F4B7BF124CC}"/>
-    <hyperlink ref="I24" r:id="rId19" xr:uid="{C76A3930-6E7E-4232-B1F1-2ED5A173BA06}"/>
-    <hyperlink ref="I22" r:id="rId20" xr:uid="{89930E83-4AEA-4DE5-8019-E1271D4CE40C}"/>
-    <hyperlink ref="I20" r:id="rId21" xr:uid="{2D3AA0A6-0D92-4AA2-9646-17F5F35EE4DB}"/>
-    <hyperlink ref="I16" r:id="rId22" xr:uid="{40199BE7-DAC8-4F2F-B423-BBE8840267EA}"/>
-    <hyperlink ref="I15" r:id="rId23" xr:uid="{35C9B14E-1DDC-4ADE-A779-D46ACC35493F}"/>
-    <hyperlink ref="I26" r:id="rId24" xr:uid="{E3724D1C-4691-4AD5-B199-6AE5E0B71D4F}"/>
-    <hyperlink ref="I13" r:id="rId25" xr:uid="{71949AF6-6BA4-468B-901F-14FEB75D0A11}"/>
-    <hyperlink ref="I27" r:id="rId26" display="https://www.ni.com/en/shop/hardware/voltage/model-ni-9221" xr:uid="{3C142A9F-BAEE-4C11-A3C2-D919604D51FF}"/>
+    <hyperlink ref="I23" r:id="rId16" xr:uid="{2332F781-0981-412B-8087-9EF083A34C09}"/>
+    <hyperlink ref="I25" r:id="rId17" xr:uid="{9D4C7BC7-8534-4598-B66B-9F4B7BF124CC}"/>
+    <hyperlink ref="I24" r:id="rId18" xr:uid="{C76A3930-6E7E-4232-B1F1-2ED5A173BA06}"/>
+    <hyperlink ref="I22" r:id="rId19" xr:uid="{89930E83-4AEA-4DE5-8019-E1271D4CE40C}"/>
+    <hyperlink ref="I20" r:id="rId20" xr:uid="{2D3AA0A6-0D92-4AA2-9646-17F5F35EE4DB}"/>
+    <hyperlink ref="I16" r:id="rId21" xr:uid="{40199BE7-DAC8-4F2F-B423-BBE8840267EA}"/>
+    <hyperlink ref="I15" r:id="rId22" xr:uid="{35C9B14E-1DDC-4ADE-A779-D46ACC35493F}"/>
+    <hyperlink ref="I26" r:id="rId23" xr:uid="{E3724D1C-4691-4AD5-B199-6AE5E0B71D4F}"/>
+    <hyperlink ref="I13" r:id="rId24" xr:uid="{71949AF6-6BA4-468B-901F-14FEB75D0A11}"/>
+    <hyperlink ref="I27" r:id="rId25" display="https://www.ni.com/en/shop/hardware/voltage/model-ni-9221" xr:uid="{3C142A9F-BAEE-4C11-A3C2-D919604D51FF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId27"/>
+  <pageSetup orientation="portrait" r:id="rId26"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
moved 2 and 4 probe boards to v0.2.1 and updated bom
</commit_message>
<xml_diff>
--- a/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
+++ b/DAQ_design/Assisi/v0.2.1/BOM-BIPHASIC-Assisi-v0.2.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Biphasic-data-acquisition-system\DAQ_design\Assisi\v0.2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9774B499-0AFA-45A0-BB82-8121C64357E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34138668-6F98-4497-ACF7-1116AA954EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="140">
   <si>
     <t>Total Cost</t>
   </si>
@@ -377,9 +377,6 @@
     <t>Cut apart and use to connect to wire mesh in concrete (slightly larger, may allow to double tap)</t>
   </si>
   <si>
-    <t>current sense resistor</t>
-  </si>
-  <si>
     <t>CPF1100K00BHB14</t>
   </si>
   <si>
@@ -408,6 +405,58 @@
   </si>
   <si>
     <t>Convenient and plugs into wall Likely will not use in the future.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 position receptical for 4 probe measurment </t>
+  </si>
+  <si>
+    <t>CPF-1 100K .1% T-2 B14</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/phoenix-contact/1757271/260477</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/phoenix-contact/1754504/260371</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/phoenix-contact/1757255/260475</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/phoenix-contact/1757022/260380</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/phoenix-contact/1786459/2526585</t>
+  </si>
+  <si>
+    <t>TERM BLOCK HDR 7POS 5.08MM</t>
+  </si>
+  <si>
+    <t>TERM BLOCK PLUG 5POS 5MM</t>
+  </si>
+  <si>
+    <t>TERM BLOCK PLUG 3POS 5.08MM</t>
+  </si>
+  <si>
+    <t>TERM BLOCK HDR 3POS 5.08MM</t>
+  </si>
+  <si>
+    <t>TERM BLOCK HDR 5POS 5.08MM</t>
+  </si>
+  <si>
+    <t>Component
+7-position connector to main board</t>
+  </si>
+  <si>
+    <t>5-position plug for 4-probe measurement</t>
+  </si>
+  <si>
+    <t>3-position receptacle for 2-probe measurement</t>
+  </si>
+  <si>
+    <t>3-position plug for 2-probe measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100k precision resistor for porbe board </t>
   </si>
 </sst>
 </file>
@@ -858,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
@@ -1438,10 +1487,10 @@
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="D19" s="2">
         <v>1</v>
@@ -1460,7 +1509,7 @@
         <v>49</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J19" s="4"/>
     </row>
@@ -1470,7 +1519,7 @@
         <v>103</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D20" s="2">
         <v>1</v>
@@ -1499,7 +1548,7 @@
         <v>70</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D21" s="8">
         <v>3</v>
@@ -1515,10 +1564,10 @@
         <v>18.600000000000001</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1767,11 +1816,14 @@
       <c r="J30" s="4"/>
     </row>
     <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="2" t="s">
+      <c r="A31" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2">
@@ -1785,82 +1837,158 @@
         <v>1.05</v>
       </c>
       <c r="H31" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="J31" s="4"/>
     </row>
     <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
+      <c r="A32" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="2">
+        <v>1786459</v>
+      </c>
       <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="7" t="s">
-        <v>10</v>
+      <c r="E32" s="2">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>7.62</v>
       </c>
       <c r="G32" s="5">
-        <f>SUM(G2:G31)</f>
-        <v>1964.8391999999999</v>
+        <f t="shared" ref="G32:G36" si="2">F32*E32</f>
+        <v>7.62</v>
       </c>
       <c r="H32" s="5"/>
-      <c r="I32" s="3"/>
+      <c r="I32" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="J32" s="4"/>
     </row>
     <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
+      <c r="A33" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="2">
+        <v>1757271</v>
+      </c>
       <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
+      <c r="E33" s="2">
+        <v>1</v>
+      </c>
+      <c r="F33" s="5">
+        <v>1.52</v>
+      </c>
+      <c r="G33" s="5">
+        <f t="shared" si="2"/>
+        <v>1.52</v>
+      </c>
       <c r="H33" s="5"/>
-      <c r="I33" s="3"/>
+      <c r="I33" s="3" t="s">
+        <v>125</v>
+      </c>
       <c r="J33" s="4"/>
     </row>
     <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
+      <c r="A34" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" s="4">
+        <v>1754504</v>
+      </c>
       <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="5"/>
+      <c r="E34" s="2">
+        <v>1</v>
+      </c>
+      <c r="F34" s="5">
+        <v>4.47</v>
+      </c>
+      <c r="G34" s="5">
+        <f t="shared" si="2"/>
+        <v>4.47</v>
+      </c>
       <c r="H34" s="5"/>
-      <c r="I34" s="3"/>
+      <c r="I34" s="3" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
+      <c r="A35" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C35" s="4">
+        <v>175725</v>
+      </c>
       <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
+      <c r="E35" s="2">
+        <v>1</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="G35" s="5">
+        <f t="shared" si="2"/>
+        <v>0.9</v>
+      </c>
       <c r="H35" s="2"/>
-      <c r="I35" s="3"/>
+      <c r="I35" s="3" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
+      <c r="A36" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36" s="4">
+        <v>1757022</v>
+      </c>
       <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
+      <c r="E36" s="2">
+        <v>1</v>
+      </c>
+      <c r="F36" s="2">
+        <v>2.71</v>
+      </c>
+      <c r="G36" s="5">
+        <f t="shared" si="2"/>
+        <v>2.71</v>
+      </c>
       <c r="H36" s="2"/>
-      <c r="I36" s="3"/>
+      <c r="I36" s="3" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
       <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F41" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" s="5">
+        <f>SUM(G2:G36)</f>
+        <v>1982.0591999999999</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1892,8 +2020,13 @@
     <hyperlink ref="I28" r:id="rId25" xr:uid="{8E893F7C-DB4B-4F4D-B291-CA255F808870}"/>
     <hyperlink ref="I31" r:id="rId26" xr:uid="{00928615-FDB1-45E3-8AB2-52E230911FE4}"/>
     <hyperlink ref="I19" r:id="rId27" xr:uid="{5AFB7500-CC61-47CA-9C71-8F739D049854}"/>
+    <hyperlink ref="I33" r:id="rId28" xr:uid="{8CF05644-1536-4813-BB61-B0DEE210F849}"/>
+    <hyperlink ref="I34" r:id="rId29" xr:uid="{9393F431-5E4B-4B6D-8840-4BC7B3FCCEB1}"/>
+    <hyperlink ref="I35" r:id="rId30" xr:uid="{F265A9C4-77A1-449B-9C65-7207AD716705}"/>
+    <hyperlink ref="I36" r:id="rId31" xr:uid="{B1A567F8-0927-48EC-8965-9D359D96BA20}"/>
+    <hyperlink ref="I32" r:id="rId32" xr:uid="{1021541E-8B31-4BB5-8D64-95533B3632C4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId28"/>
+  <pageSetup orientation="portrait" r:id="rId33"/>
 </worksheet>
 </file>
</xml_diff>